<commit_message>
Final copy of theory
</commit_message>
<xml_diff>
--- a/Theory.xlsx
+++ b/Theory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git_June_22\project1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CAC3300-D973-47A0-8EBD-023D553EA16B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B587225-6FD4-4DE6-851A-86E18B07BBC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{28229DAC-A180-4F0F-87B8-08E9AB6A9375}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="43">
   <si>
     <t>Initially</t>
   </si>
@@ -115,13 +115,61 @@
   </si>
   <si>
     <t>switch to feature</t>
+  </si>
+  <si>
+    <t>main</t>
+  </si>
+  <si>
+    <t>fea1</t>
+  </si>
+  <si>
+    <t>Rebase</t>
+  </si>
+  <si>
+    <t>Main</t>
+  </si>
+  <si>
+    <t>file1</t>
+  </si>
+  <si>
+    <t>line 5</t>
+  </si>
+  <si>
+    <t>some code</t>
+  </si>
+  <si>
+    <t>Feature</t>
+  </si>
+  <si>
+    <t>some other code</t>
+  </si>
+  <si>
+    <t>PR &amp; merge</t>
+  </si>
+  <si>
+    <t>git  checkout main</t>
+  </si>
+  <si>
+    <t>merge main - feature1</t>
+  </si>
+  <si>
+    <t>push to remote</t>
+  </si>
+  <si>
+    <t>changes in feature1</t>
+  </si>
+  <si>
+    <t>personal project</t>
+  </si>
+  <si>
+    <t>prod project</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -134,6 +182,12 @@
       <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1463,6 +1517,300 @@
           <a:r>
             <a:rPr lang="en-IN" sz="1100" baseline="0"/>
             <a:t> local</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-IN" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>130</xdr:row>
+      <xdr:rowOff>177800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>137</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="19" name="Oval 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7389BCA5-59A2-39E7-CFD5-F8D4585C1C47}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5562600" y="24168100"/>
+          <a:ext cx="1238250" cy="1136650"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-IN" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>317500</xdr:colOff>
+      <xdr:row>132</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>138</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="20" name="TextBox 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E6E7C494-1991-B0DB-7500-223651CC24B3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5803900" y="24377650"/>
+          <a:ext cx="768350" cy="1098550"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100"/>
+            <a:t>main</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-IN" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100"/>
+            <a:t>file1</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100"/>
+            <a:t>modified f1</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-IN" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>215900</xdr:colOff>
+      <xdr:row>138</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
+      <xdr:row>146</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="21" name="Oval 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{05273A40-01A2-2505-D0E2-B54377EBD766}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5702300" y="25628600"/>
+          <a:ext cx="1377950" cy="1447800"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-IN" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>469900</xdr:colOff>
+      <xdr:row>140</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>139700</xdr:colOff>
+      <xdr:row>145</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="22" name="TextBox 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{10B813FF-720D-2E0E-335E-A6825B9414E8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5956300" y="25933400"/>
+          <a:ext cx="889000" cy="876300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100"/>
+            <a:t>feature 1</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-IN" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100"/>
+            <a:t>file1</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100"/>
+            <a:t>modified</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" baseline="0"/>
+            <a:t> f1</a:t>
           </a:r>
           <a:endParaRPr lang="en-IN" sz="1100"/>
         </a:p>
@@ -1770,7 +2118,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D244690-24BE-427E-945E-87DC4EE9CADC}">
-  <dimension ref="C34:G135"/>
+  <dimension ref="B34:L135"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="34" spans="4:7" x14ac:dyDescent="0.35">
@@ -1867,7 +2215,75 @@
         <v>17</v>
       </c>
     </row>
-    <row r="125" spans="3:6" x14ac:dyDescent="0.35">
+    <row r="102" spans="4:12" x14ac:dyDescent="0.35">
+      <c r="D102" t="s">
+        <v>29</v>
+      </c>
+      <c r="L102" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="103" spans="4:12" x14ac:dyDescent="0.35">
+      <c r="L103" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="104" spans="4:12" x14ac:dyDescent="0.35">
+      <c r="L104" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="105" spans="4:12" x14ac:dyDescent="0.35">
+      <c r="D105" t="s">
+        <v>30</v>
+      </c>
+      <c r="L105" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="106" spans="4:12" x14ac:dyDescent="0.35">
+      <c r="D106" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="107" spans="4:12" x14ac:dyDescent="0.35">
+      <c r="D107" t="s">
+        <v>32</v>
+      </c>
+      <c r="E107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L107" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="108" spans="4:12" x14ac:dyDescent="0.35">
+      <c r="H108" t="s">
+        <v>36</v>
+      </c>
+      <c r="L108" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="109" spans="4:12" x14ac:dyDescent="0.35">
+      <c r="D109" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="110" spans="4:12" x14ac:dyDescent="0.35">
+      <c r="D110" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="111" spans="4:12" x14ac:dyDescent="0.35">
+      <c r="D111" t="s">
+        <v>32</v>
+      </c>
+      <c r="E111" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="125" spans="2:6" x14ac:dyDescent="0.35">
       <c r="C125" t="s">
         <v>18</v>
       </c>
@@ -1875,7 +2291,10 @@
         <v>20</v>
       </c>
     </row>
-    <row r="126" spans="3:6" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B126" t="s">
+        <v>27</v>
+      </c>
       <c r="C126" t="s">
         <v>19</v>
       </c>
@@ -1883,7 +2302,18 @@
         <v>21</v>
       </c>
     </row>
-    <row r="128" spans="3:6" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B127" t="s">
+        <v>28</v>
+      </c>
+      <c r="C127" t="s">
+        <v>19</v>
+      </c>
+      <c r="F127" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="128" spans="2:6" x14ac:dyDescent="0.35">
       <c r="E128" t="s">
         <v>22</v>
       </c>
@@ -1914,6 +2344,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>